<commit_message>
thana no fixed in village
</commit_message>
<xml_diff>
--- a/uploads/excels/LIMS_Test_Pvt_land_Data_format_24.03.26_(1)_(2).xlsx
+++ b/uploads/excels/LIMS_Test_Pvt_land_Data_format_24.03.26_(1)_(2).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\lims up file format\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maasuser\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44D2F5D8-2374-40DC-951B-7CCB3C09BA99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB8F33E0-EFBF-46FE-9184-FDFD7EB66FA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,21 +24,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="696" uniqueCount="299">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="696" uniqueCount="301">
   <si>
     <t>SES Survey No.</t>
   </si>
@@ -936,6 +927,12 @@
   </si>
   <si>
     <t>demand of higher compensation</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>N</t>
   </si>
 </sst>
 </file>
@@ -2155,7 +2152,7 @@
         <v>282</v>
       </c>
       <c r="CF2" s="11" t="s">
-        <v>252</v>
+        <v>299</v>
       </c>
     </row>
     <row r="3" spans="1:86" ht="62.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2395,7 +2392,7 @@
         <v>282</v>
       </c>
       <c r="CF3" s="11" t="s">
-        <v>252</v>
+        <v>300</v>
       </c>
     </row>
     <row r="4" spans="1:86" ht="45" x14ac:dyDescent="0.25">
@@ -2628,7 +2625,7 @@
         <v>282</v>
       </c>
       <c r="CF4" s="11" t="s">
-        <v>252</v>
+        <v>299</v>
       </c>
     </row>
     <row r="5" spans="1:86" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2852,7 +2849,7 @@
         <v>281</v>
       </c>
       <c r="CF5" s="11" t="s">
-        <v>268</v>
+        <v>300</v>
       </c>
       <c r="CG5" s="55">
         <v>46102</v>
@@ -3056,7 +3053,7 @@
         <v>281</v>
       </c>
       <c r="CF6" s="11" t="s">
-        <v>268</v>
+        <v>299</v>
       </c>
       <c r="CG6" s="55">
         <v>46102</v>
@@ -3269,7 +3266,7 @@
         <v>281</v>
       </c>
       <c r="CF7" s="11" t="s">
-        <v>268</v>
+        <v>300</v>
       </c>
       <c r="CG7" s="55">
         <v>46102</v>
@@ -4126,7 +4123,7 @@
         <v>286</v>
       </c>
       <c r="CF15" s="8" t="s">
-        <v>268</v>
+        <v>299</v>
       </c>
       <c r="CG15" s="44">
         <v>46106</v>
@@ -4290,7 +4287,7 @@
         <v>286</v>
       </c>
       <c r="CF16" s="8" t="s">
-        <v>268</v>
+        <v>300</v>
       </c>
       <c r="CG16" s="44">
         <v>46106</v>

</xml_diff>